<commit_message>
Gộp dữ liệu 26/10 (5 kênh đủ, TGDD thiếu mảnh 3) + post_sync: gộp ngay kênh đã xong khi còn pending
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zjvRAgpUXc2uYHGJpjNs5
</commit_message>
<xml_diff>
--- a/laptop_gearvn_all.xlsx
+++ b/laptop_gearvn_all.xlsx
@@ -45,7 +45,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -53,13 +53,19 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -540,7 +546,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:19:55</t>
+          <t>2026-10-26 00:13:29</t>
         </is>
       </c>
     </row>
@@ -584,7 +590,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:01</t>
+          <t>2026-10-26 00:13:34</t>
         </is>
       </c>
     </row>
@@ -628,7 +634,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:06</t>
+          <t>2026-10-26 00:13:39</t>
         </is>
       </c>
     </row>
@@ -672,7 +678,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:11</t>
+          <t>2026-10-26 00:13:44</t>
         </is>
       </c>
     </row>
@@ -716,7 +722,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:16</t>
+          <t>2026-10-26 00:13:49</t>
         </is>
       </c>
     </row>
@@ -760,7 +766,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:21</t>
+          <t>2026-10-26 00:13:54</t>
         </is>
       </c>
     </row>
@@ -804,7 +810,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:27</t>
+          <t>2026-10-26 00:13:59</t>
         </is>
       </c>
     </row>
@@ -848,7 +854,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:32</t>
+          <t>2026-10-26 00:14:04</t>
         </is>
       </c>
     </row>
@@ -892,7 +898,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:38</t>
+          <t>2026-10-26 00:14:09</t>
         </is>
       </c>
     </row>
@@ -936,7 +942,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:43</t>
+          <t>2026-10-26 00:14:14</t>
         </is>
       </c>
     </row>
@@ -980,7 +986,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:48</t>
+          <t>2026-10-26 00:14:19</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1030,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:53</t>
+          <t>2026-10-26 00:14:25</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1074,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:58</t>
+          <t>2026-10-26 00:14:29</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1118,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:03</t>
+          <t>2026-10-26 00:14:35</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1162,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:08</t>
+          <t>2026-10-26 00:14:40</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1206,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:13</t>
+          <t>2026-10-26 00:14:45</t>
         </is>
       </c>
     </row>
@@ -1211,14 +1217,14 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>19890000</v>
+        <v>19990000</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>19990000</v>
+        <v>24990000</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>-1%</t>
+          <t>-20%</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1244,7 +1250,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:18</t>
+          <t>2026-10-26 00:14:50</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1294,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:23</t>
+          <t>2026-10-26 00:14:55</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1332,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:29</t>
+          <t>2026-10-26 00:15:00</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1370,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:34</t>
+          <t>2026-10-26 00:15:06</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1414,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:39</t>
+          <t>2026-10-26 00:15:11</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1452,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:44</t>
+          <t>2026-10-26 00:15:16</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1496,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:50</t>
+          <t>2026-10-26 00:15:21</t>
         </is>
       </c>
     </row>
@@ -1501,14 +1507,14 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>29390000</v>
+        <v>29790000</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>29790000</v>
+        <v>30990000</v>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>-1%</t>
+          <t>-4%</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1534,7 +1540,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:55</t>
+          <t>2026-10-26 00:15:26</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1584,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:00</t>
+          <t>2026-10-26 00:15:31</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1628,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:05</t>
+          <t>2026-10-26 00:15:37</t>
         </is>
       </c>
     </row>
@@ -1660,7 +1666,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:10</t>
+          <t>2026-10-26 00:15:42</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1710,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:16</t>
+          <t>2026-10-26 00:15:47</t>
         </is>
       </c>
     </row>
@@ -1748,7 +1754,7 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:21</t>
+          <t>2026-10-26 00:15:52</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1798,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:26</t>
+          <t>2026-10-26 00:15:57</t>
         </is>
       </c>
     </row>
@@ -1836,7 +1842,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:31</t>
+          <t>2026-10-26 00:16:02</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1886,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:36</t>
+          <t>2026-10-26 00:16:07</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1926,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:42</t>
+          <t>2026-10-26 00:16:13</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1970,7 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:47</t>
+          <t>2026-10-26 00:16:18</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2014,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:52</t>
+          <t>2026-10-26 00:16:23</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2058,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:57</t>
+          <t>2026-10-26 00:16:28</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2102,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:02</t>
+          <t>2026-10-26 00:16:33</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2142,7 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:07</t>
+          <t>2026-10-26 00:16:38</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2186,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:12</t>
+          <t>2026-10-26 00:16:44</t>
         </is>
       </c>
     </row>
@@ -2220,7 +2226,7 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:17</t>
+          <t>2026-10-26 00:16:49</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2266,7 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:23</t>
+          <t>2026-10-26 00:16:54</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2306,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:28</t>
+          <t>2026-10-26 00:17:00</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2350,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:34</t>
+          <t>2026-10-26 00:17:05</t>
         </is>
       </c>
     </row>
@@ -2388,7 +2394,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:39</t>
+          <t>2026-10-26 00:17:10</t>
         </is>
       </c>
     </row>
@@ -2432,7 +2438,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:18</t>
+          <t>2026-10-26 00:13:30</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2476,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:23</t>
+          <t>2026-10-26 00:13:35</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2514,7 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:28</t>
+          <t>2026-10-26 00:13:41</t>
         </is>
       </c>
     </row>
@@ -2546,7 +2552,7 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:33</t>
+          <t>2026-10-26 00:13:46</t>
         </is>
       </c>
     </row>
@@ -2584,7 +2590,7 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:38</t>
+          <t>2026-10-26 00:13:51</t>
         </is>
       </c>
     </row>
@@ -2628,7 +2634,7 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:43</t>
+          <t>2026-10-26 00:13:56</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2672,7 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:48</t>
+          <t>2026-10-26 00:14:01</t>
         </is>
       </c>
     </row>
@@ -2704,7 +2710,7 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:54</t>
+          <t>2026-10-26 00:14:06</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2754,7 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:58</t>
+          <t>2026-10-26 00:14:11</t>
         </is>
       </c>
     </row>
@@ -2786,7 +2792,7 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:03</t>
+          <t>2026-10-26 00:14:16</t>
         </is>
       </c>
     </row>
@@ -2820,7 +2826,7 @@
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:08</t>
+          <t>2026-10-26 00:14:21</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2860,7 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:14</t>
+          <t>2026-10-26 00:14:26</t>
         </is>
       </c>
     </row>
@@ -2892,7 +2898,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:19</t>
+          <t>2026-10-26 00:14:31</t>
         </is>
       </c>
     </row>
@@ -2930,7 +2936,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:24</t>
+          <t>2026-10-26 00:14:36</t>
         </is>
       </c>
     </row>
@@ -2968,7 +2974,7 @@
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:29</t>
+          <t>2026-10-26 00:14:41</t>
         </is>
       </c>
     </row>
@@ -3006,7 +3012,7 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:34</t>
+          <t>2026-10-26 00:14:47</t>
         </is>
       </c>
     </row>
@@ -3044,7 +3050,7 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:39</t>
+          <t>2026-10-26 00:14:52</t>
         </is>
       </c>
     </row>
@@ -3082,7 +3088,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:44</t>
+          <t>2026-10-26 00:14:57</t>
         </is>
       </c>
     </row>
@@ -3120,7 +3126,7 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:49</t>
+          <t>2026-10-26 00:15:02</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3164,7 @@
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:54</t>
+          <t>2026-10-26 00:15:07</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3202,7 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:58</t>
+          <t>2026-10-26 00:15:12</t>
         </is>
       </c>
     </row>
@@ -3234,7 +3240,7 @@
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:03</t>
+          <t>2026-10-26 00:15:17</t>
         </is>
       </c>
     </row>
@@ -3272,7 +3278,7 @@
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:08</t>
+          <t>2026-10-26 00:15:22</t>
         </is>
       </c>
     </row>
@@ -3316,7 +3322,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:13</t>
+          <t>2026-10-26 00:15:27</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3360,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:18</t>
+          <t>2026-10-26 00:15:32</t>
         </is>
       </c>
     </row>
@@ -3392,7 +3398,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:23</t>
+          <t>2026-10-26 00:15:37</t>
         </is>
       </c>
     </row>
@@ -3436,7 +3442,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:28</t>
+          <t>2026-10-26 00:15:42</t>
         </is>
       </c>
     </row>
@@ -3474,7 +3480,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:34</t>
+          <t>2026-10-26 00:15:47</t>
         </is>
       </c>
     </row>
@@ -3512,7 +3518,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:39</t>
+          <t>2026-10-26 00:15:52</t>
         </is>
       </c>
     </row>
@@ -3550,7 +3556,7 @@
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:44</t>
+          <t>2026-10-26 00:15:57</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3594,7 @@
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:49</t>
+          <t>2026-10-26 00:16:03</t>
         </is>
       </c>
     </row>
@@ -3626,7 +3632,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:54</t>
+          <t>2026-10-26 00:16:08</t>
         </is>
       </c>
     </row>
@@ -3664,7 +3670,7 @@
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:59</t>
+          <t>2026-10-26 00:16:13</t>
         </is>
       </c>
     </row>
@@ -3702,7 +3708,7 @@
       </c>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:04</t>
+          <t>2026-10-26 00:16:18</t>
         </is>
       </c>
     </row>
@@ -3740,7 +3746,7 @@
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:09</t>
+          <t>2026-10-26 00:16:23</t>
         </is>
       </c>
     </row>
@@ -3778,7 +3784,7 @@
       </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:14</t>
+          <t>2026-10-26 00:16:28</t>
         </is>
       </c>
     </row>
@@ -3822,7 +3828,7 @@
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:19</t>
+          <t>2026-10-26 00:16:33</t>
         </is>
       </c>
     </row>
@@ -3866,7 +3872,7 @@
       </c>
       <c r="J83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:24</t>
+          <t>2026-10-26 00:16:38</t>
         </is>
       </c>
     </row>
@@ -3906,7 +3912,7 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:29</t>
+          <t>2026-10-26 00:16:43</t>
         </is>
       </c>
     </row>
@@ -3950,7 +3956,7 @@
       </c>
       <c r="J85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:34</t>
+          <t>2026-10-26 00:16:48</t>
         </is>
       </c>
     </row>
@@ -3994,7 +4000,7 @@
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:39</t>
+          <t>2026-10-26 00:16:53</t>
         </is>
       </c>
     </row>
@@ -4034,7 +4040,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:44</t>
+          <t>2026-10-26 00:16:58</t>
         </is>
       </c>
     </row>
@@ -4078,7 +4084,7 @@
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:49</t>
+          <t>2026-10-26 00:17:04</t>
         </is>
       </c>
     </row>
@@ -4116,7 +4122,7 @@
       </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:54</t>
+          <t>2026-10-26 00:17:09</t>
         </is>
       </c>
     </row>
@@ -4160,7 +4166,7 @@
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:19:53</t>
+          <t>2026-10-26 00:13:20</t>
         </is>
       </c>
     </row>
@@ -4171,14 +4177,14 @@
         </is>
       </c>
       <c r="B91" s="3" t="n">
-        <v>24790000</v>
+        <v>24990000</v>
       </c>
       <c r="C91" s="2" t="n">
-        <v>24990000</v>
+        <v>27990000</v>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>-1%</t>
+          <t>-11%</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -4204,7 +4210,7 @@
       </c>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:19:59</t>
+          <t>2026-10-26 00:13:26</t>
         </is>
       </c>
     </row>
@@ -4248,7 +4254,7 @@
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:05</t>
+          <t>2026-10-26 00:13:31</t>
         </is>
       </c>
     </row>
@@ -4292,7 +4298,7 @@
       </c>
       <c r="J93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:10</t>
+          <t>2026-10-26 00:13:36</t>
         </is>
       </c>
     </row>
@@ -4330,7 +4336,7 @@
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:15</t>
+          <t>2026-10-26 00:13:41</t>
         </is>
       </c>
     </row>
@@ -4374,7 +4380,7 @@
       </c>
       <c r="J95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:20</t>
+          <t>2026-10-26 00:13:46</t>
         </is>
       </c>
     </row>
@@ -4418,7 +4424,7 @@
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:25</t>
+          <t>2026-10-26 00:13:51</t>
         </is>
       </c>
     </row>
@@ -4429,14 +4435,14 @@
         </is>
       </c>
       <c r="B97" s="3" t="n">
-        <v>32990000</v>
+        <v>33290000</v>
       </c>
       <c r="C97" s="2" t="n">
-        <v>33290000</v>
+        <v>34990000</v>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>-1%</t>
+          <t>-5%</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -4462,7 +4468,7 @@
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:30</t>
+          <t>2026-10-26 00:13:56</t>
         </is>
       </c>
     </row>
@@ -4506,7 +4512,7 @@
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:35</t>
+          <t>2026-10-26 00:14:01</t>
         </is>
       </c>
     </row>
@@ -4517,16 +4523,10 @@
         </is>
       </c>
       <c r="B99" s="3" t="n">
-        <v>37990000</v>
-      </c>
-      <c r="C99" s="2" t="n">
         <v>38990000</v>
       </c>
-      <c r="D99" s="2" t="inlineStr">
-        <is>
-          <t>-3%</t>
-        </is>
-      </c>
+      <c r="C99" s="2" t="inlineStr"/>
+      <c r="D99" s="2" t="inlineStr"/>
       <c r="E99" s="2" t="inlineStr">
         <is>
           <t>Tặng ngay 1 x Màn hình Acer KG241Y-X1 24" IPS 200Hz Gsync chuyên game (trị giá 2.390.000đ) | Tặng ngay 1 x Balo Acer Predator SUV (trị giá 2.000.000đ)</t>
@@ -4550,7 +4550,7 @@
       </c>
       <c r="J99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:40</t>
+          <t>2026-10-26 00:14:06</t>
         </is>
       </c>
     </row>
@@ -4594,7 +4594,7 @@
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:46</t>
+          <t>2026-10-26 00:14:11</t>
         </is>
       </c>
     </row>
@@ -4632,7 +4632,7 @@
       </c>
       <c r="J101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:51</t>
+          <t>2026-10-26 00:14:16</t>
         </is>
       </c>
     </row>
@@ -4670,7 +4670,7 @@
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:56</t>
+          <t>2026-10-26 00:14:21</t>
         </is>
       </c>
     </row>
@@ -4708,7 +4708,7 @@
       </c>
       <c r="J103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:01</t>
+          <t>2026-10-26 00:14:26</t>
         </is>
       </c>
     </row>
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:06</t>
+          <t>2026-10-26 00:14:31</t>
         </is>
       </c>
     </row>
@@ -4790,7 +4790,7 @@
       </c>
       <c r="J105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:11</t>
+          <t>2026-10-26 00:14:36</t>
         </is>
       </c>
     </row>
@@ -4834,7 +4834,7 @@
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:16</t>
+          <t>2026-10-26 00:14:41</t>
         </is>
       </c>
     </row>
@@ -4878,7 +4878,7 @@
       </c>
       <c r="J107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:21</t>
+          <t>2026-10-26 00:14:46</t>
         </is>
       </c>
     </row>
@@ -4916,7 +4916,7 @@
       </c>
       <c r="J108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:26</t>
+          <t>2026-10-26 00:14:51</t>
         </is>
       </c>
     </row>
@@ -4960,7 +4960,7 @@
       </c>
       <c r="J109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:31</t>
+          <t>2026-10-26 00:14:56</t>
         </is>
       </c>
     </row>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:36</t>
+          <t>2026-10-26 00:15:01</t>
         </is>
       </c>
     </row>
@@ -5048,7 +5048,7 @@
       </c>
       <c r="J111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:42</t>
+          <t>2026-10-26 00:15:06</t>
         </is>
       </c>
     </row>
@@ -5092,7 +5092,7 @@
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:47</t>
+          <t>2026-10-26 00:15:11</t>
         </is>
       </c>
     </row>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:52</t>
+          <t>2026-10-26 00:15:16</t>
         </is>
       </c>
     </row>
@@ -5180,7 +5180,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:57</t>
+          <t>2026-10-26 00:15:21</t>
         </is>
       </c>
     </row>
@@ -5224,7 +5224,7 @@
       </c>
       <c r="J115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:02</t>
+          <t>2026-10-26 00:15:27</t>
         </is>
       </c>
     </row>
@@ -5268,7 +5268,7 @@
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:07</t>
+          <t>2026-10-26 00:15:32</t>
         </is>
       </c>
     </row>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:12</t>
+          <t>2026-10-26 00:15:37</t>
         </is>
       </c>
     </row>
@@ -5344,7 +5344,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:17</t>
+          <t>2026-10-26 00:15:42</t>
         </is>
       </c>
     </row>
@@ -5382,7 +5382,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:22</t>
+          <t>2026-10-26 00:15:47</t>
         </is>
       </c>
     </row>
@@ -5426,7 +5426,7 @@
       </c>
       <c r="J120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:28</t>
+          <t>2026-10-26 00:15:52</t>
         </is>
       </c>
     </row>
@@ -5466,7 +5466,7 @@
       </c>
       <c r="J121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:33</t>
+          <t>2026-10-26 00:15:57</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:38</t>
+          <t>2026-10-26 00:16:02</t>
         </is>
       </c>
     </row>
@@ -5544,7 +5544,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:43</t>
+          <t>2026-10-26 00:16:07</t>
         </is>
       </c>
     </row>
@@ -5588,7 +5588,7 @@
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:48</t>
+          <t>2026-10-26 00:16:12</t>
         </is>
       </c>
     </row>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="J125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:53</t>
+          <t>2026-10-26 00:16:17</t>
         </is>
       </c>
     </row>
@@ -5664,7 +5664,7 @@
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:58</t>
+          <t>2026-10-26 00:16:22</t>
         </is>
       </c>
     </row>
@@ -5702,7 +5702,7 @@
       </c>
       <c r="J127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:03</t>
+          <t>2026-10-26 00:16:27</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:08</t>
+          <t>2026-10-26 00:16:32</t>
         </is>
       </c>
     </row>
@@ -5780,7 +5780,7 @@
       </c>
       <c r="J129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:13</t>
+          <t>2026-10-26 00:16:37</t>
         </is>
       </c>
     </row>
@@ -5824,7 +5824,7 @@
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:18</t>
+          <t>2026-10-26 00:16:43</t>
         </is>
       </c>
     </row>
@@ -5862,7 +5862,7 @@
       </c>
       <c r="J131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:23</t>
+          <t>2026-10-26 00:16:48</t>
         </is>
       </c>
     </row>
@@ -5906,7 +5906,7 @@
       </c>
       <c r="J132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:29</t>
+          <t>2026-10-26 00:16:53</t>
         </is>
       </c>
     </row>
@@ -5944,7 +5944,7 @@
       </c>
       <c r="J133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:34</t>
+          <t>2026-10-26 00:16:57</t>
         </is>
       </c>
     </row>
@@ -5978,7 +5978,7 @@
       </c>
       <c r="J134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:19:42</t>
+          <t>2026-10-26 00:13:29</t>
         </is>
       </c>
     </row>
@@ -6016,7 +6016,7 @@
       </c>
       <c r="J135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:19:47</t>
+          <t>2026-10-26 00:13:35</t>
         </is>
       </c>
     </row>
@@ -6050,7 +6050,7 @@
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:19:53</t>
+          <t>2026-10-26 00:13:40</t>
         </is>
       </c>
     </row>
@@ -6084,7 +6084,7 @@
       </c>
       <c r="J137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:19:57</t>
+          <t>2026-10-26 00:13:45</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:02</t>
+          <t>2026-10-26 00:13:50</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:07</t>
+          <t>2026-10-26 00:13:56</t>
         </is>
       </c>
     </row>
@@ -6198,7 +6198,7 @@
       </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:13</t>
+          <t>2026-10-26 00:14:01</t>
         </is>
       </c>
     </row>
@@ -6236,7 +6236,7 @@
       </c>
       <c r="J141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:18</t>
+          <t>2026-10-26 00:14:06</t>
         </is>
       </c>
     </row>
@@ -6274,7 +6274,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:23</t>
+          <t>2026-10-26 00:14:11</t>
         </is>
       </c>
     </row>
@@ -6312,7 +6312,7 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:28</t>
+          <t>2026-10-26 00:14:16</t>
         </is>
       </c>
     </row>
@@ -6350,7 +6350,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:33</t>
+          <t>2026-10-26 00:14:21</t>
         </is>
       </c>
     </row>
@@ -6388,7 +6388,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:38</t>
+          <t>2026-10-26 00:14:26</t>
         </is>
       </c>
     </row>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:43</t>
+          <t>2026-10-26 00:14:31</t>
         </is>
       </c>
     </row>
@@ -6476,7 +6476,7 @@
       </c>
       <c r="J147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:48</t>
+          <t>2026-10-26 00:14:36</t>
         </is>
       </c>
     </row>
@@ -6520,7 +6520,7 @@
       </c>
       <c r="J148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:53</t>
+          <t>2026-10-26 00:14:41</t>
         </is>
       </c>
     </row>
@@ -6564,7 +6564,7 @@
       </c>
       <c r="J149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:58</t>
+          <t>2026-10-26 00:14:46</t>
         </is>
       </c>
     </row>
@@ -6604,7 +6604,7 @@
       </c>
       <c r="J150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:03</t>
+          <t>2026-10-26 00:14:51</t>
         </is>
       </c>
     </row>
@@ -6644,7 +6644,7 @@
       </c>
       <c r="J151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:08</t>
+          <t>2026-10-26 00:14:57</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:13</t>
+          <t>2026-10-26 00:15:02</t>
         </is>
       </c>
     </row>
@@ -6732,7 +6732,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:18</t>
+          <t>2026-10-26 00:15:07</t>
         </is>
       </c>
     </row>
@@ -6770,7 +6770,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:23</t>
+          <t>2026-10-26 00:15:12</t>
         </is>
       </c>
     </row>
@@ -6808,7 +6808,7 @@
       </c>
       <c r="J155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:28</t>
+          <t>2026-10-26 00:15:17</t>
         </is>
       </c>
     </row>
@@ -6846,7 +6846,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:33</t>
+          <t>2026-10-26 00:15:22</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6884,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:38</t>
+          <t>2026-10-26 00:15:28</t>
         </is>
       </c>
     </row>
@@ -6922,7 +6922,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:43</t>
+          <t>2026-10-26 00:15:33</t>
         </is>
       </c>
     </row>
@@ -6966,7 +6966,7 @@
       </c>
       <c r="J159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:48</t>
+          <t>2026-10-26 00:15:38</t>
         </is>
       </c>
     </row>
@@ -7010,7 +7010,7 @@
       </c>
       <c r="J160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:53</t>
+          <t>2026-10-26 00:15:43</t>
         </is>
       </c>
     </row>
@@ -7054,7 +7054,7 @@
       </c>
       <c r="J161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:58</t>
+          <t>2026-10-26 00:15:49</t>
         </is>
       </c>
     </row>
@@ -7098,7 +7098,7 @@
       </c>
       <c r="J162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:03</t>
+          <t>2026-10-26 00:15:54</t>
         </is>
       </c>
     </row>
@@ -7109,14 +7109,14 @@
         </is>
       </c>
       <c r="B163" s="3" t="n">
-        <v>29790000</v>
+        <v>29990000</v>
       </c>
       <c r="C163" s="2" t="n">
-        <v>29990000</v>
+        <v>30990000</v>
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>-1%</t>
+          <t>-3%</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
@@ -7142,7 +7142,7 @@
       </c>
       <c r="J163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:08</t>
+          <t>2026-10-26 00:15:59</t>
         </is>
       </c>
     </row>
@@ -7153,14 +7153,14 @@
         </is>
       </c>
       <c r="B164" s="3" t="n">
-        <v>31790000</v>
+        <v>31990000</v>
       </c>
       <c r="C164" s="2" t="n">
-        <v>31990000</v>
+        <v>34990000</v>
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>-1%</t>
+          <t>-9%</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
@@ -7186,7 +7186,7 @@
       </c>
       <c r="J164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:13</t>
+          <t>2026-10-26 00:16:04</t>
         </is>
       </c>
     </row>
@@ -7230,7 +7230,7 @@
       </c>
       <c r="J165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:18</t>
+          <t>2026-10-26 00:16:09</t>
         </is>
       </c>
     </row>
@@ -7274,7 +7274,7 @@
       </c>
       <c r="J166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:23</t>
+          <t>2026-10-26 00:16:14</t>
         </is>
       </c>
     </row>
@@ -7318,7 +7318,7 @@
       </c>
       <c r="J167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:28</t>
+          <t>2026-10-26 00:16:19</t>
         </is>
       </c>
     </row>
@@ -7356,7 +7356,7 @@
       </c>
       <c r="J168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:33</t>
+          <t>2026-10-26 00:16:24</t>
         </is>
       </c>
     </row>
@@ -7400,7 +7400,7 @@
       </c>
       <c r="J169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:38</t>
+          <t>2026-10-26 00:16:29</t>
         </is>
       </c>
     </row>
@@ -7444,7 +7444,7 @@
       </c>
       <c r="J170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:43</t>
+          <t>2026-10-26 00:16:34</t>
         </is>
       </c>
     </row>
@@ -7488,7 +7488,7 @@
       </c>
       <c r="J171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:48</t>
+          <t>2026-10-26 00:16:39</t>
         </is>
       </c>
     </row>
@@ -7526,7 +7526,7 @@
       </c>
       <c r="J172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:53</t>
+          <t>2026-10-26 00:16:44</t>
         </is>
       </c>
     </row>
@@ -7564,7 +7564,7 @@
       </c>
       <c r="J173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:58</t>
+          <t>2026-10-26 00:16:49</t>
         </is>
       </c>
     </row>
@@ -7608,7 +7608,7 @@
       </c>
       <c r="J174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:02</t>
+          <t>2026-10-26 00:16:55</t>
         </is>
       </c>
     </row>
@@ -7652,7 +7652,7 @@
       </c>
       <c r="J175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:08</t>
+          <t>2026-10-26 00:17:00</t>
         </is>
       </c>
     </row>
@@ -7690,7 +7690,7 @@
       </c>
       <c r="J176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:13</t>
+          <t>2026-10-26 00:17:05</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="J177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:18</t>
+          <t>2026-10-26 00:17:10</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="J178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:00</t>
+          <t>2026-10-26 00:13:40</t>
         </is>
       </c>
     </row>
@@ -7810,7 +7810,7 @@
       </c>
       <c r="J179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:05</t>
+          <t>2026-10-26 00:13:46</t>
         </is>
       </c>
     </row>
@@ -7848,7 +7848,7 @@
       </c>
       <c r="J180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:10</t>
+          <t>2026-10-26 00:13:52</t>
         </is>
       </c>
     </row>
@@ -7892,7 +7892,7 @@
       </c>
       <c r="J181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:15</t>
+          <t>2026-10-26 00:13:56</t>
         </is>
       </c>
     </row>
@@ -7936,7 +7936,7 @@
       </c>
       <c r="J182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:20</t>
+          <t>2026-10-26 00:14:01</t>
         </is>
       </c>
     </row>
@@ -7974,7 +7974,7 @@
       </c>
       <c r="J183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:25</t>
+          <t>2026-10-26 00:14:06</t>
         </is>
       </c>
     </row>
@@ -8012,7 +8012,7 @@
       </c>
       <c r="J184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:30</t>
+          <t>2026-10-26 00:14:11</t>
         </is>
       </c>
     </row>
@@ -8050,7 +8050,7 @@
       </c>
       <c r="J185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:35</t>
+          <t>2026-10-26 00:14:16</t>
         </is>
       </c>
     </row>
@@ -8084,7 +8084,7 @@
       </c>
       <c r="J186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:40</t>
+          <t>2026-10-26 00:14:22</t>
         </is>
       </c>
     </row>
@@ -8118,7 +8118,7 @@
       </c>
       <c r="J187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:45</t>
+          <t>2026-10-26 00:14:27</t>
         </is>
       </c>
     </row>
@@ -8158,7 +8158,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:50</t>
+          <t>2026-10-26 00:14:32</t>
         </is>
       </c>
     </row>
@@ -8198,7 +8198,7 @@
       </c>
       <c r="J189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:20:56</t>
+          <t>2026-10-26 00:14:37</t>
         </is>
       </c>
     </row>
@@ -8236,7 +8236,7 @@
       </c>
       <c r="J190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:01</t>
+          <t>2026-10-26 00:14:42</t>
         </is>
       </c>
     </row>
@@ -8274,7 +8274,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:06</t>
+          <t>2026-10-26 00:14:47</t>
         </is>
       </c>
     </row>
@@ -8312,7 +8312,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:11</t>
+          <t>2026-10-26 00:14:52</t>
         </is>
       </c>
     </row>
@@ -8350,7 +8350,7 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:16</t>
+          <t>2026-10-26 00:14:57</t>
         </is>
       </c>
     </row>
@@ -8388,7 +8388,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:21</t>
+          <t>2026-10-26 00:15:02</t>
         </is>
       </c>
     </row>
@@ -8422,7 +8422,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:26</t>
+          <t>2026-10-26 00:15:07</t>
         </is>
       </c>
     </row>
@@ -8460,7 +8460,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:31</t>
+          <t>2026-10-26 00:15:12</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:36</t>
+          <t>2026-10-26 00:15:17</t>
         </is>
       </c>
     </row>
@@ -8536,7 +8536,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:41</t>
+          <t>2026-10-26 00:15:22</t>
         </is>
       </c>
     </row>
@@ -8574,7 +8574,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:46</t>
+          <t>2026-10-26 00:15:27</t>
         </is>
       </c>
     </row>
@@ -8618,7 +8618,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:51</t>
+          <t>2026-10-26 00:15:33</t>
         </is>
       </c>
     </row>
@@ -8639,9 +8639,17 @@
           <t>-3%</t>
         </is>
       </c>
-      <c r="E201" s="2" t="inlineStr"/>
+      <c r="E201" s="2" t="inlineStr">
+        <is>
+          <t>[Laptop] Giảm 1% tối đa 500k cho HSSV khi mua laptop</t>
+        </is>
+      </c>
       <c r="F201" s="2" t="inlineStr"/>
-      <c r="G201" s="2" t="inlineStr"/>
+      <c r="G201" s="2" t="inlineStr">
+        <is>
+          <t>Card đồ họa: Intel Graphics | Kích thước màn hình: 16 inch | Dòng CPU: Core Ultra 5 | Dung lượng SSD: 512 GB | Tấm nền: IPS | Độ phân giải: 2K+ (2560x1600) | Dung lượng RAM: 16 GB</t>
+        </is>
+      </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
           <t>https://gearvn.com/products/laptop-lg-gram-pro-16z90u-g-an55a5-ultra-5-325-16gb-512gb-16-0-wqxga-win-11</t>
@@ -8654,7 +8662,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:21:56</t>
+          <t>2026-10-26 00:15:38</t>
         </is>
       </c>
     </row>
@@ -8675,9 +8683,17 @@
           <t>-3%</t>
         </is>
       </c>
-      <c r="E202" s="2" t="inlineStr"/>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>[Laptop] Giảm 1% tối đa 500k cho HSSV khi mua laptop</t>
+        </is>
+      </c>
       <c r="F202" s="2" t="inlineStr"/>
-      <c r="G202" s="2" t="inlineStr"/>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>Card đồ họa: Intel Graphics | Kích thước màn hình: 16 inch | Dòng CPU: Core Ultra 7 | Dung lượng SSD: 512 GB | Tấm nền: IPS | Độ phân giải: 2K+ (2560x1600) | Dung lượng RAM: 32 GB</t>
+        </is>
+      </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
           <t>https://gearvn.com/products/laptop-lg-gram-pro-16z90u-g-av85a5-ultra-7-355-32gb-512gb-intel-graphics-16-0-wqxga-win-11</t>
@@ -8690,7 +8706,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:01</t>
+          <t>2026-10-26 00:15:43</t>
         </is>
       </c>
     </row>
@@ -8734,7 +8750,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:06</t>
+          <t>2026-10-26 00:15:48</t>
         </is>
       </c>
     </row>
@@ -8778,7 +8794,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:11</t>
+          <t>2026-10-26 00:15:53</t>
         </is>
       </c>
     </row>
@@ -8822,7 +8838,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:16</t>
+          <t>2026-10-26 00:15:58</t>
         </is>
       </c>
     </row>
@@ -8862,7 +8878,7 @@
       </c>
       <c r="J206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:21</t>
+          <t>2026-10-26 00:16:03</t>
         </is>
       </c>
     </row>
@@ -8900,7 +8916,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:26</t>
+          <t>2026-10-26 00:16:08</t>
         </is>
       </c>
     </row>
@@ -8944,7 +8960,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:31</t>
+          <t>2026-10-26 00:16:13</t>
         </is>
       </c>
     </row>
@@ -8988,7 +9004,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:37</t>
+          <t>2026-10-26 00:16:18</t>
         </is>
       </c>
     </row>
@@ -9032,7 +9048,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:42</t>
+          <t>2026-10-26 00:16:23</t>
         </is>
       </c>
     </row>
@@ -9076,7 +9092,7 @@
       </c>
       <c r="J211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:47</t>
+          <t>2026-10-26 00:16:28</t>
         </is>
       </c>
     </row>
@@ -9120,7 +9136,7 @@
       </c>
       <c r="J212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:52</t>
+          <t>2026-10-26 00:16:33</t>
         </is>
       </c>
     </row>
@@ -9154,7 +9170,7 @@
       </c>
       <c r="J213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:22:57</t>
+          <t>2026-10-26 00:16:38</t>
         </is>
       </c>
     </row>
@@ -9169,7 +9185,11 @@
       </c>
       <c r="C214" s="2" t="inlineStr"/>
       <c r="D214" s="2" t="inlineStr"/>
-      <c r="E214" s="2" t="inlineStr"/>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t>[Laptop] Giảm 1% tối đa 500k cho HSSV khi mua laptop</t>
+        </is>
+      </c>
       <c r="F214" s="2" t="inlineStr"/>
       <c r="G214" s="2" t="inlineStr"/>
       <c r="H214" s="2" t="inlineStr">
@@ -9184,7 +9204,7 @@
       </c>
       <c r="J214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:02</t>
+          <t>2026-10-26 00:16:43</t>
         </is>
       </c>
     </row>
@@ -9218,7 +9238,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:07</t>
+          <t>2026-10-26 00:16:49</t>
         </is>
       </c>
     </row>
@@ -9252,7 +9272,7 @@
       </c>
       <c r="J216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:12</t>
+          <t>2026-10-26 00:16:54</t>
         </is>
       </c>
     </row>
@@ -9296,7 +9316,7 @@
       </c>
       <c r="J217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:17</t>
+          <t>2026-10-26 00:16:59</t>
         </is>
       </c>
     </row>
@@ -9340,7 +9360,7 @@
       </c>
       <c r="J218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25 00:23:23</t>
+          <t>2026-10-26 00:17:04</t>
         </is>
       </c>
     </row>

</xml_diff>